<commit_message>
[feat] MatchStrategyData 전투 행동 선택 가중치 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/MatchStrategyData.xlsx
+++ b/JsonConverter/ExcelFiles/MatchStrategyData.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="28545" windowHeight="11745"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="28545" windowHeight="13035"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <x:si>
     <x:t>레슬링위주 공격적 압박</x:t>
   </x:si>
@@ -27,64 +27,82 @@
     <x:t>스탠딩위주 공격적 압박</x:t>
   </x:si>
   <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>strategy_02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>후반을 바라보기</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SortOrder</x:t>
+  </x:si>
+  <x:si>
+    <x:t>strategy_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>strategy_00</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IsDefault</x:t>
+  </x:si>
+  <x:si>
+    <x:t>strategy_03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>상대와 비교하는 행동 선택률</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float</x:t>
+  </x:si>
+  <x:si>
+    <x:t>기본 운영</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
     <x:t>(name)</x:t>
   </x:si>
   <x:si>
     <x:t>bool</x:t>
   </x:si>
   <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
     <x:t>Name</x:t>
   </x:si>
   <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
+    <x:t>후반 라운드를 생각하며 체력을 보존한다. 스태미너 소모를 줄이고 가벼운 공격만 하며 라운드 점수 따기 위주 운영을 한다.</x:t>
   </x:si>
   <x:si>
     <x:t>스탠딩 상황에서 상대의 주의를 끌 큰 공격들을 던지며 테이크다운을 노린다. 거세게 압박하여 스태미너 소모를 많이 한다.</x:t>
   </x:si>
   <x:si>
-    <x:t>후반 라운드를 생각하며 체력을 보존한다. 스태미너 소모를 줄이고 가벼운 공격만 하며 라운드 점수 따기 위주 운영을 한다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>strategy_00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IsDefault</x:t>
-  </x:si>
-  <x:si>
-    <x:t>strategy_03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SortOrder</x:t>
-  </x:si>
-  <x:si>
-    <x:t>후반을 바라보기</x:t>
-  </x:si>
-  <x:si>
-    <x:t>strategy_02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>strategy_01</x:t>
-  </x:si>
-  <x:si>
     <x:t>상대를 케이지에 몰아넣으며 스탠딩 타격 위주로 거친 압박을 가한다.</x:t>
   </x:si>
   <x:si>
-    <x:t>기본 운영</x:t>
-  </x:si>
-  <x:si>
     <x:t>특별한 지시 없이 기존 경기 운영을 유지한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WrestlingSelectionWeight</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JiuJitsuSelectionWeight</x:t>
+  </x:si>
+  <x:si>
+    <x:t>StrikeSelectionWeight</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ActionSelectionWeight</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -855,70 +873,98 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:H35"/>
+  <x:dimension ref="A1:I35"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="25.4296875" style="1" customWidth="1"/>
     <x:col min="2" max="2" width="24.71484375" style="1" customWidth="1"/>
     <x:col min="3" max="3" width="65.4296875" style="1" customWidth="1"/>
-    <x:col min="4" max="6" width="20.26953125" style="1" customWidth="1"/>
+    <x:col min="4" max="5" width="20.26953125" style="1" customWidth="1"/>
+    <x:col min="6" max="6" width="25.4296875" style="1" customWidth="1"/>
     <x:col min="7" max="7" width="30.54296875" style="1" customWidth="1"/>
     <x:col min="8" max="8" width="26.54296875" style="1" customWidth="1"/>
-    <x:col min="9" max="9" width="20" style="1" customWidth="1"/>
+    <x:col min="9" max="9" width="23.4296875" style="1" customWidth="1"/>
     <x:col min="10" max="12" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
     <x:col min="13" max="13" width="15.71484375" style="1" customWidth="1"/>
     <x:col min="14" max="14" width="17.4296875" style="1" customWidth="1"/>
     <x:col min="15" max="16384" width="12.54296875" style="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5" ht="13.199999999999999">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:9" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="I2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:9" s="7" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="2" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
+      <x:c r="D3" s="7" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E3" s="7" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5" s="7" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="2" t="s">
+      <x:c r="F3" s="7" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G3" s="7" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="H3" s="7" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="I3" s="7" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:9" ht="15.75" customHeight="1">
+      <x:c r="A4" s="3" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="7" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="D3" s="7" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="E3" s="7" t="s">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:8" ht="15.75" customHeight="1">
-      <x:c r="A4" s="3" t="s">
-        <x:v>11</x:v>
-      </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>20</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C4" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D4" s="1" t="b">
         <x:v>1</x:v>
@@ -926,17 +972,28 @@
       <x:c r="E4" s="1">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H4" s="4"/>
-    </x:row>
-    <x:row r="5" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F4" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G4" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H4" s="4">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I4" s="1">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:9" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="1" t="b">
         <x:v>0</x:v>
@@ -944,16 +1001,28 @@
       <x:c r="E5" s="1">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F5" s="1">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="G5" s="1">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H5" s="1">
+        <x:v>0.59999999999999998</x:v>
+      </x:c>
+      <x:c r="I5" s="1">
+        <x:v>0.59999999999999998</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:9" ht="15.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>17</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D6" s="1" t="b">
         <x:v>0</x:v>
@@ -961,22 +1030,46 @@
       <x:c r="E6" s="1">
         <x:v>2</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" spans="1:5" ht="15.75" customHeight="1">
+      <x:c r="F6" s="1">
+        <x:v>1.3</x:v>
+      </x:c>
+      <x:c r="G6" s="1">
+        <x:v>0.59999999999999998</x:v>
+      </x:c>
+      <x:c r="H6" s="1">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I6" s="1">
+        <x:v>0.80000000000000004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:9" ht="15.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
-        <x:v>14</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>16</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C7" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D7" s="1" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="1">
         <x:v>3</x:v>
+      </x:c>
+      <x:c r="F7" s="1">
+        <x:v>0.69999999999999996</x:v>
+      </x:c>
+      <x:c r="G7" s="1">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H7" s="1">
+        <x:v>0.69999999999999996</x:v>
+      </x:c>
+      <x:c r="I7" s="1">
+        <x:v>0.69999999999999996</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:2" ht="15.75" customHeight="1">

</xml_diff>